<commit_message>
publish live hog price report 2026-07-22
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_2026-07-22.xlsx
+++ b/reports/越南生猪价格省级三大区_2026-07-22.xlsx
@@ -669,15 +669,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -690,403 +689,353 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>来源表省份明细；价格单位为VND/kg。中文省名用于阅读，越南语原名保留用于复核。</t>
+          <t>来源表省份明细；价格单位为VND/kg。首列为中文省份，越南语原名保留用于复核。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>序号</t>
+          <t>省份（中文）</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>省份（中文）</t>
+          <t>省份（越南语）</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>省份（越南语）</t>
+          <t>价格（VND/kg）</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>价格（VND/kg）</t>
+          <t>增加/减少（VND）</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>增加/减少（VND）</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>宣光</t>
+        </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>宣光</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
           <t>Tuyên Quang</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>2</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>高平</t>
+        </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>高平</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
           <t>Cao Bằng</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>太原</t>
+        </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>太原</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
           <t>Thái Nguyên</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="D7" s="9" t="n">
         <v>-1000</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>下降</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>4</v>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>谅山</t>
+        </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>谅山</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
           <t>Lạng Sơn</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="C8" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>5</v>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>广宁</t>
+        </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>广宁</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
           <t>Quảng Ninh</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>6</v>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>北宁</t>
+        </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>北宁</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
           <t>Bắc Ninh</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="C10" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>7</v>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>河内</t>
+        </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>河内</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
           <t>Hà Nội</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="C11" s="6" t="n">
         <v>67000</v>
       </c>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>8</v>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>海防</t>
+        </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>海防</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
           <t>Hải Phòng</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="C12" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="5" t="n">
-        <v>9</v>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>宁平</t>
+        </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>宁平</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
           <t>Ninh Bình</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>10</v>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>老街</t>
+        </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>老街</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
           <t>Lào Cai</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="C14" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="5" t="n">
-        <v>11</v>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>莱州</t>
+        </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>莱州</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
           <t>Lai Châu</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="C15" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="D15" s="9" t="n">
         <v>-1000</v>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>下降</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="5" t="n">
-        <v>12</v>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>奠边</t>
+        </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>奠边</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
           <t>Điện Biên</t>
         </is>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="C16" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="5" t="n">
-        <v>13</v>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>富寿</t>
+        </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>富寿</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
           <t>Phú Thọ</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="C17" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="5" t="n">
-        <v>14</v>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>山罗</t>
+        </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>山罗</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
           <t>Sơn La</t>
         </is>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="D18" s="9" t="n">
         <v>-1000</v>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>下降</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="5" t="n">
-        <v>15</v>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>兴安</t>
+        </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>兴安</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
           <t>Hưng Yên</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="C19" s="6" t="n">
         <v>67000</v>
       </c>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
@@ -1094,8 +1043,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1107,15 +1056,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1128,301 +1076,263 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>来源表省份明细；价格单位为VND/kg。中文省名用于阅读，越南语原名保留用于复核。</t>
+          <t>来源表省份明细；价格单位为VND/kg。首列为中文省份，越南语原名保留用于复核。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>序号</t>
+          <t>省份（中文）</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>省份（中文）</t>
+          <t>省份（越南语）</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>省份（越南语）</t>
+          <t>价格（VND/kg）</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>价格（VND/kg）</t>
+          <t>增加/减少（VND）</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>增加/减少（VND）</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>清化</t>
+        </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>清化</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
           <t>Thanh Hoá</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>2</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>乂安</t>
+        </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>乂安</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
           <t>Nghệ An</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>河静</t>
+        </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>河静</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
           <t>Hà Tĩnh</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>4</v>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>广治</t>
+        </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>广治</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
           <t>Quảng Trị</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="C8" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>5</v>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>顺化</t>
+        </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>顺化</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
           <t>Huế</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>6</v>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>岘港</t>
+        </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>岘港</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
           <t>Đà Nẵng</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>7</v>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>广义</t>
+        </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广义</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
           <t>Quảng Ngãi</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>8</v>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>嘉莱</t>
+        </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>嘉莱</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
           <t>Gia Lai</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="5" t="n">
-        <v>9</v>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>得乐</t>
+        </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>得乐</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
           <t>Đắk Lắk</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>10</v>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>庆和</t>
+        </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>庆和</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
           <t>Khánh Hoà</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="5" t="n">
-        <v>11</v>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>林同</t>
+        </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>林同</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
           <t>Lâm Đồng</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="C15" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
@@ -1430,8 +1340,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1443,15 +1353,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1464,229 +1373,200 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>来源表省份明细；价格单位为VND/kg。中文省名用于阅读，越南语原名保留用于复核。</t>
+          <t>来源表省份明细；价格单位为VND/kg。首列为中文省份，越南语原名保留用于复核。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>序号</t>
+          <t>省份（中文）</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>省份（中文）</t>
+          <t>省份（越南语）</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>省份（越南语）</t>
+          <t>价格（VND/kg）</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>价格（VND/kg）</t>
+          <t>增加/减少（VND）</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>增加/减少（VND）</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>同奈</t>
+        </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>同奈</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
           <t>Đồng Nai</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>2</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>西宁</t>
+        </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>西宁</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
           <t>Tây Ninh</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>同塔</t>
+        </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>同塔</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
           <t>Đồng Tháp</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>4</v>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>安江</t>
+        </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>安江</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
           <t>An Giang</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>5</v>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>金瓯</t>
+        </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>金瓯</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
           <t>Cà Mau</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>6</v>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市</t>
+        </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
           <t>TP HCM</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>7</v>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>永隆</t>
+        </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>永隆</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
           <t>Vĩnh Long</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>8</v>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>芹苴</t>
+        </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>芹苴</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
           <t>Cần Thơ</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
         </is>
@@ -1694,8 +1574,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>